<commit_message>
lf09: update asset statuses, add PASTE_BRIEF.md
</commit_message>
<xml_diff>
--- a/longform/lf09-australia-full/assets-list/lf09_Asset_List.xlsx
+++ b/longform/lf09-australia-full/assets-list/lf09_Asset_List.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Not held in any prior film (lf03/lf05 logged ParlView as FREE SWAP). Reuse-only rule: not downloaded. Fallback: Hansard quote card only.</t>
+          <t>FREE SWAP per script; Not held in any prior film (lf03/lf05 logged ParlView as FREE SWAP). Reuse-only rule: not downloaded. Fallback: Hansard quote card only.</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Not held previously. Fallback: date card + Senate chamber still (lf05 IMG-senate-chamber.jpg, JJ Harrison CC BY-SA 3.0) — not copied.</t>
+          <t>FREE SWAP per script; Not held previously. Fallback: date card + Senate chamber still (lf05 IMG-senate-chamber.jpg, JJ Harrison CC BY-SA 3.0) — not copied.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Not held previously. Fallback: Farrer map + name card.</t>
+          <t>FREE SWAP per script; Not held previously. Fallback: Farrer map + name card.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>FREE SWAP (no new ParlView). Fallback: IMG_burke + E12 card.</t>
+          <t>FREE SWAP per script; FREE SWAP (no new ParlView). Fallback: IMG_burke + E12 card.</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>FREE SWAP (no new ParlView). Fallback: IMG_haines + paraphrase card.</t>
+          <t>FREE SWAP per script; FREE SWAP (no new ParlView). Fallback: IMG_haines + paraphrase card.</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,6 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1035,7 +1034,6 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1415,32 +1413,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>footage/stock/BR_STOCK_airport_arrivals_board.mp4</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pexels/Pixabay search</t>
+          <t>https://www.pexels.com/video/low-angle-view-of-flight-schedules-on-a-board-4684084/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pexels License</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Taryn Elliott</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>no faceless free clip found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Pexels, supplied by user 15 Oct</t>
         </is>
       </c>
     </row>
@@ -1452,32 +1450,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>footage/stock/BR_STOCK_rental_inspection_keys.mp4</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Pexels/Pixabay search</t>
+          <t>https://www.pexels.com/video/hand-holding-keys-over-money-and-mini-house-model-31400388/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pexels License</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Jakub Zerdzicki</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Mixkit keys clips show faces; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Pexels, supplied by user 15 Oct</t>
         </is>
       </c>
     </row>
@@ -1489,32 +1487,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>footage/stock/BR_STOCK_hospital_corridor_empty.mp4</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Pexels/Pixabay search</t>
+          <t>https://www.pexels.com/video/an-empty-hospital-hallway-5203510/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pexels License</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Enrique Silva</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>none found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Pexels, supplied by user 15 Oct</t>
         </is>
       </c>
     </row>
@@ -1526,32 +1524,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>footage/stock/BR_STOCK_nurse_corridor_back.mp4</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pexels/Pixabay search</t>
+          <t>https://www.pexels.com/video/medical-worker-walking-in-the-hallway-8381605/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pexels License</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pavel Danilyuk</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>none found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Pexels, supplied by user 15 Oct</t>
         </is>
       </c>
     </row>
@@ -1563,32 +1561,32 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>footage/stock/BR_STOCK_apartment_cranes.mp4</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pexels/Pixabay search</t>
+          <t>https://www.pexels.com/video/high-rise-construction-with-cranes-38871857/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pexels License</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Kiwi and Camera</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Mixkit cranes clip is Restricted licence; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Pexels, supplied by user 15 Oct</t>
         </is>
       </c>
     </row>
@@ -1600,32 +1598,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>footage/stock/BR_STOCK_passport_desk_generic.mp4</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Pexels/Pixabay search</t>
+          <t>https://www.pexels.com/video/passport-on-top-of-a-laptop-7308237/</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pexels License</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RDNE Stock project</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>none checked faceless; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Pexels, supplied by user 15 Oct (mp4, script ID was .jpg)</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1660,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>none found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Script fallback: regional map / IMG_haines + card</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1697,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>none found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Script fallback: Parliament House stock / BR_AI_election_night_empty_hall</t>
         </is>
       </c>
     </row>
@@ -1711,32 +1709,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>footage/stock/BR_STOCK_lecture_hall_empty.mp4</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Pexels/Pixabay search</t>
+          <t>https://www.pexels.com/video/an-empty-classroom-8342689/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pexels License</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pavel Danilyuk</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>none found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Pexels, supplied by user 15 Oct</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1771,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Mixkit results show faces; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Script fallback: BR_STOCK_university_campus_aerial / lecture hall</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1808,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>none found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Script fallback: regional map + name/paraphrase card</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1845,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>none found; Pexels/Pixabay need a browser download — fetch manually or use a still/AI stand-in</t>
+          <t>Script fallback: regional map + card</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1857,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>broll/BR_AI_canberra_dawn_fog.mp4</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Grok Imagine (broll/AI_PROMPTS.tsv)</t>
+          <t>Grok Imagine</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1874,17 +1872,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI-generated (Grok Imagine)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>To generate; not made here</t>
+          <t>720p, 10 s, Grok watermark bottom-right: crop/cover</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1894,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>broll/BR_AI_outback_aerial_empty.mp4</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Grok Imagine (broll/AI_PROMPTS.tsv)</t>
+          <t>Grok Imagine</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1911,17 +1909,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI-generated (Grok Imagine)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>To generate; not made here</t>
+          <t>720p, 10 s, Grok watermark bottom-right: crop/cover</t>
         </is>
       </c>
     </row>
@@ -1933,12 +1931,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>broll/BR_AI_1990s_lounge_tv_glow.mp4</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Grok Imagine (broll/AI_PROMPTS.tsv)</t>
+          <t>Grok Imagine</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1948,17 +1946,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI-generated (Grok Imagine)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>To generate; not made here</t>
+          <t>720p, 10 s, Grok watermark bottom-right: crop/cover</t>
         </is>
       </c>
     </row>
@@ -1970,12 +1968,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>broll/BR_AI_election_night_empty_hall.mp4</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Grok Imagine (broll/AI_PROMPTS.tsv)</t>
+          <t>Grok Imagine</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1985,17 +1983,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI-generated (Grok Imagine)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>To generate; not made here</t>
+          <t>720p, 10 s, Grok watermark bottom-right: crop/cover</t>
         </is>
       </c>
     </row>
@@ -2007,12 +2005,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>broll/BR_AI_cafe_empty_morning.mp4</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Grok Imagine (broll/AI_PROMPTS.tsv)</t>
+          <t>Grok Imagine</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2022,17 +2020,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI-generated (Grok Imagine)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>To generate; not made here</t>
+          <t>720p, 10 s, Grok watermark bottom-right: crop/cover</t>
         </is>
       </c>
     </row>
@@ -2044,12 +2042,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>broll/BR_AI_strategy_room_whiteboard.mp4</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Grok Imagine (broll/AI_PROMPTS.tsv)</t>
+          <t>Grok Imagine</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2059,17 +2057,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI-generated (Grok Imagine)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>To generate; not made here</t>
+          <t>720p, 10 s, Grok watermark bottom-right: crop/cover</t>
         </is>
       </c>
     </row>
@@ -2081,12 +2079,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>broll/BR_AI_thumbnail_bg.png</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Grok Imagine (broll/AI_PROMPTS.tsv)</t>
+          <t>Grok Imagine</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2096,17 +2094,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI-generated (Grok Imagine)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>To generate; not made here</t>
+          <t>Rough, garbled text; optional</t>
         </is>
       </c>
     </row>
@@ -2414,32 +2412,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_slot_roll.mp3</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/film-special-effects-slot-machine-reels-sound-30276/</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>freesound_community</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2451,32 +2449,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_split_flap.mp3</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/city-split-flap-display-58766/</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>freesound_community</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2599,32 +2597,32 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_thread_snap.mp3</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/film-special-effects-rope-sound-effect-272812/</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>soundreality</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2710,32 +2708,32 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_chain_rattle.mp3</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/film-special-effects-chain-6073/</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>freesound_community</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2747,32 +2745,32 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_padlock_break.mp3</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/household-locked-door-being-forced-open-85088/</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>freesound_community</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2784,32 +2782,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_receipt_printer.mp3</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/technology-receipt-printer-01-43872/</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>freesound_community</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2895,32 +2893,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_heartbeat.mp3</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/film-special-effects-heartbeat-sound-372448/</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dragon Studio</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2932,32 +2930,32 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_lamp_click.mp3</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/household-light-switch-382712/</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dragon Studio</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -2969,32 +2967,32 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_glass_clink.mp3</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/film-special-effects-glass-clink-57538/</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>freesound_community</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -3006,32 +3004,32 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_drone_low.mp3</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/film-special-effects-deep-haunting-drone-482880/</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dragon Studio</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>
@@ -3043,32 +3041,32 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>audio/sfx/SFX_room_tone.mp3</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Pixabay / Freesound CC0</t>
+          <t>https://pixabay.com/sound-effects/film-special-effects-room-tone-42-74466/</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pixabay Content License</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>freesound_community</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>MISSING-fallback</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Pixabay/Freesound downloads need browser/login; fetch manually</t>
+          <t>Pixabay, supplied by user 15 Oct (mp3)</t>
         </is>
       </c>
     </row>

</xml_diff>